<commit_message>
feat(mappings): add sbe-orchestra mappings to model
</commit_message>
<xml_diff>
--- a/project/excel/fix_orchestra.xlsx
+++ b/project/excel/fix_orchestra.xlsx
@@ -163,6 +163,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="154" state="visible" r:id="rId154"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sections" sheetId="155" state="visible" r:id="rId155"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="156" state="visible" r:id="rId156"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIXMLencodingType" sheetId="157" state="visible" r:id="rId157"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4687,6 +4688,32 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet157.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>inlined</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>not_req_xml</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -8120,7 +8147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8146,75 +8173,80 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>fixml_encoding</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>lang_id</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>purpose</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>added</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>added_ep</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>change_type</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>deprecated_ep</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>issue</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>last_modified</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>replaced</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>replaced_ep</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>replaced_by_field</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>supported</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>updated</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>updated_ep</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>deprecated</t>
         </is>
@@ -8222,10 +8254,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Editorial,Definitional"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"supported,forbidden,ignored"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>